<commit_message>
Ajout bouton lien vers dashboard Power BI
</commit_message>
<xml_diff>
--- a/data/besoins_production.xlsx
+++ b/data/besoins_production.xlsx
@@ -5,15 +5,15 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/58830f9fc3ba735f/Documents/pilotage-stock-production/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\israc\OneDrive\Documents\pilotage-stock-production\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_2B59D2BFD300DD8AB9495A33469528F06A3DFB0E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D111D67-8C96-4F06-8017-AC5B025456F1}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C048D428-2514-4DB8-9AB0-D00A36BF86FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="besoin production" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>

</xml_diff>